<commit_message>
Draft interview setup workbook: day template and availability grid
Proposed standard format for interview events, for review before the import
is rebuilt around it: Event (with minimum panel size), Day template (blocks
of interviews, breaks and calibration by duration), Judges, Availability
(one row per judge, one column per date and block; Yes, No/blank, or a
24-hour window like 13:00-16:00), optional Candidates and Criteria.

The API's workbook reader still expects the earlier per-session Schedule
format, so this branch is not deployable until the import follows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qkgbu6zx8nSF6qinJQFGfA
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/event-setup-template.xlsx
+++ b/apps/web/public/templates/event-setup-template.xlsx
@@ -9,10 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rooms" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judges" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day template" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judges" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Availability" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -22,9 +22,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="hh:mm"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="hh:mm"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -97,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -116,7 +115,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -201,12 +199,12 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Where the event happens, e.g. Asia/Singapore. All times on the Schedule are in this timezone. Default Asia/Singapore.</t>
+        <t>Where the interviews happen, e.g. Asia/Singapore. Every time in this workbook is in this timezone. Default Asia/Singapore.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>The usual length of a judging session. Each Schedule row still has its own start and end.</t>
+        <t>Fewest judges an interview needs. Slots with fewer available judges are left without a panel. Default 2.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -226,12 +224,17 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Must be unique. The Schedule refers to rooms by this name.</t>
+        <t>A name for the half-day block, e.g. AM or PM. The Availability sheet uses the same names.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>24-hour HH:MM. Only on the first row of each block; the rest follow on one after another.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Y if a team can present by video in this room.</t>
+        <t>Interview, Break or Calibration.</t>
       </text>
     </comment>
   </commentList>
@@ -244,24 +247,19 @@
     <author>Template</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Must be unique. The Schedule refers to teams by this name.</t>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>Must be unique. The Availability sheet refers to judges by email.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Tracks are created from this column.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>2-letter code, e.g. SG</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>In person or Video. Default In person.</t>
+        <t>With country code, e.g. +6591234567</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional label: L1, L2, L3, L4, PS or V.</t>
       </text>
     </comment>
   </commentList>
@@ -274,19 +272,29 @@
     <author>Template</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Exactly as on the Judges sheet.</t>
+      </text>
+    </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Must be unique. The Schedule refers to judges by email.</t>
+        <t>Yes, No, or a window like 13:00-16:00</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>With country code, e.g. +6591234567</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional label: L1, L2, L3, L4, PS or V.</t>
+        <t>Yes, No, or a window like 13:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Yes, No, or a window like 13:00-16:00</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Yes, No, or a window like 13:00-16:00</t>
       </text>
     </comment>
   </commentList>
@@ -301,32 +309,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>YYYY-MM-DD, or an Excel date. 12/10/2026 style dates are refused: they read differently in different countries.</t>
-      </text>
-    </comment>
-    <comment ref="B1" authorId="0" shapeId="0">
-      <text>
-        <t>24-hour HH:MM, in the event's timezone.</t>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0">
-      <text>
-        <t>24-hour HH:MM.</t>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0">
-      <text>
-        <t>Exactly as on the Rooms sheet.</t>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0">
-      <text>
-        <t>Exactly as on the Teams sheet. Each team appears once.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Exactly as on the Judges sheet.</t>
+        <t>Must be unique. Optional sheet: candidates can also be added in the app later.</t>
       </text>
     </comment>
   </commentList>
@@ -657,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -666,14 +649,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Event setup workbook</t>
+          <t>Interview setup workbook</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in every sheet and upload this file under Upload setup. The upload checks everything first, shows you what it will create, and only builds the event when you confirm. It then opens the Command Centre.</t>
+          <t>Fill in the sheets and upload this file under Upload setup. The upload checks everything first and shows the schedule it will build. Nothing is saved until you confirm.</t>
         </is>
       </c>
     </row>
@@ -683,145 +666,118 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>How to fill it in</t>
+          <t>How it works</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Dark blue header = required column. Light blue header = optional. Hover a header for notes.</t>
+          <t>Day template describes one day: each block (AM, PM) is a run of interviews, breaks and calibration with their lengths. Every judging day uses it.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Yellow rows are examples. Overwrite or delete them before uploading.</t>
+          <t>Availability says which judges can sit which block on which date. The system builds every day's slots from the template and seats each judge in the interviews they are available for.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Keep the sheet names and column headers as they are.</t>
+          <t>One panel interviews at a time. Interviews with fewer judges than the minimum panel size are left without a panel and shown greyed out.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Dates as YYYY-MM-DD (2026-10-12). Times as 24-hour HH:MM (09:30), in the event's timezone.</t>
+          <t>Candidates are placed into interview slots afterwards, on the Schedule page.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>The Schedule refers to rooms, teams and judges by name / email exactly as written on their own sheets.</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Availability format (the only accepted entries)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Sheets</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Yes = available for the whole block.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Event: one row describing the event.</t>
+          <t>No, or blank = not available.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Rooms: one row per judging room.</t>
+          <t>HH:MM-HH:MM in 24-hour time, e.g. 13:00-16:00 = available only within that window. The judge sits only the interviews that fit entirely inside it.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Teams: one row per team. Tracks are created from the Track column.</t>
+          <t>Anything else stops the upload and is listed with the judge and column so it can be corrected.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Judges: one row per judge. Email identifies the judge and must be unique.</t>
+          <t>Column headers on the Availability sheet are the date and block: YYYY-MM-DD AM, YYYY-MM-DD PM. Add one column per date and block; dates with no judges simply stay empty.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Schedule: one row per judging session. Each team appears once. The judging days are the dates used here.</t>
-        </is>
-      </c>
+      <c r="A16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Criteria (optional): the scoring rubric. Leave it empty to use the standard UOB rubric.</t>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>How to fill it in</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Dark blue header = required column. Light blue header = optional. Hover a header for notes.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>What blocks an upload</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Yellow cells are examples. Overwrite or delete them before uploading.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>An empty required cell; a room, team or judge on the Schedule that isn't on its own sheet; a team scheduled twice; a judge or room booked twice at overlapping times; an end time not after the start; duplicate team names or judge emails; a rubric that doesn't add up.</t>
+          <t>Keep the sheet names and column headers as they are. Times are 24-hour HH:MM.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>What only warns</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>A session with one judge; a video team in a room without video conferencing; a judge with more than 8 sessions in a day; teams, judges or rooms that aren't used; admin emails without a login.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Uploading again</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>You can upload a corrected file for the same event until the first score is entered. It replaces the whole setup.</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Candidates and Criteria are optional. With no Criteria, the standard UOB rubric is used.</t>
         </is>
       </c>
     </row>
@@ -842,7 +798,7 @@
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -862,9 +818,9 @@
           <t>Timezone</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Session length (minutes) *</t>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Minimum panel size</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
@@ -876,7 +832,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>UOB Innovation Challenge 2026</t>
+          <t>UOB Interviews October 2026</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
@@ -890,7 +846,7 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
@@ -910,69 +866,397 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Room name *</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Video conferencing</t>
+          <t>Block *</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Start time *</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Item *</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Duration (minutes) *</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Room A</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Level 12</t>
-        </is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>0.375</v>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Room B</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Level 12</t>
-        </is>
-      </c>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n"/>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Break</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.5833333333333334</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Break</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Interview</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Calibration</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Y,N"</formula1>
+    <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Interview,Break,Calibration"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -981,194 +1265,6 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Team name *</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Project name *</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Track</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Country</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Organisation</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Team lead name *</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Team lead email *</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>Presentation mode</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>Problem statement</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>Solution summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Team Alpha</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Smart Onboarding</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>Customer Experience</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>UOB Singapore</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>Tan Wei Ling</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>weiling@example.com</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>In person</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>Account opening takes 3 days.</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>Guided digital onboarding with document OCR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Team Beta</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Fraud Radar</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>MY</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>UOB Malaysia</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Ahmad Faiz</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>faiz@example.com</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>Card fraud is detected too late.</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>Real-time anomaly scoring on transactions.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="H2:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"In person,Video"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1220,12 +1316,12 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Lim Chee Keong</t>
+          <t>Dean Tan</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>cheekeong@example.com</t>
+          <t>dean@example.com</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -1252,12 +1348,12 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Priya Nair</t>
+          <t>Lawrance Lim</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>priya@example.com</t>
+          <t>lawrance@example.com</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -1284,12 +1380,12 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Daniel Wong</t>
+          <t>Choon Hin Ong</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>daniel@example.com</t>
+          <t>choonhin@example.com</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -1304,19 +1400,154 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Senior Engineer</t>
+          <t>Director</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>L3</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"L1,L2,L3,L4,PS,V"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Judge email *</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19 AM</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-19 PM</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20 AM</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-20 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>dean@example.com</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>lawrance@example.com</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>13:00-16:00</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>choonhin@example.com</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1330,144 +1561,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Date *</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Start time *</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>End time *</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Room *</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Team name *</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Judge 1 email *</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Judge 2 email</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
-        <is>
-          <t>Judge 3 email</t>
-        </is>
-      </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>Judge 4 email</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>Judge 5 email</t>
+          <t>Candidate name *</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>Role applied for</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="n">
-        <v>46307</v>
-      </c>
-      <c r="B2" s="8" t="n">
-        <v>0.3958333333333333</v>
-      </c>
-      <c r="C2" s="8" t="n">
-        <v>0.4131944444444444</v>
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Candidate One</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>c1@example.com</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>+6580000001</t>
+        </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Room A</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Team Alpha</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>cheekeong@example.com</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>priya@example.com</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>daniel@example.com</t>
-        </is>
-      </c>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B3" s="8" t="n">
-        <v>0.3958333333333333</v>
-      </c>
-      <c r="C3" s="8" t="n">
-        <v>0.4131944444444444</v>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Candidate Two</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>c2@example.com</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>+6580000002</t>
+        </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Room B</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>Team Beta</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>cheekeong@example.com</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>priya@example.com</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>daniel@example.com</t>
-        </is>
-      </c>
+          <t>Analyst</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1520,7 +1695,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Web: setup preview, interview schedule with drag and drop, candidate upload
Upload setup previews the schedule the workbook builds: days, blocks, how
many interviews have a panel, and who sits. The Schedule page shows upload
events as an interview schedule: day tabs with fill counts, each block's
interviews, break and calibration, panels per interview. Candidates are
dragged onto another slot (dropping on a filled one swaps) or moved to
another day with Move to; started interviews can't be moved. A day's panels
can be locked. Upload candidates checks a candidates file and shows adds and
moves before placing them.

Templates: event-setup-template.xlsx and candidates-template.xlsx, both
generated by tools/setup-workbook/build.py with a 10-day sample event and two
candidate batches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qkgbu6zx8nSF6qinJQFGfA
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/event-setup-template.xlsx
+++ b/apps/web/public/templates/event-setup-template.xlsx
@@ -12,8 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day template" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judges" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Availability" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -302,21 +301,6 @@
 </file>
 
 <file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Template</author>
-  </authors>
-  <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Must be unique. Optional sheet: candidates can also be added in the app later.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -694,7 +678,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Candidates are placed into interview slots afterwards, on the Schedule page.</t>
+          <t>Candidates are not in this workbook. Once the schedule exists, upload them in batches with the candidates file (Name, Date, Time), as they confirm.</t>
         </is>
       </c>
     </row>
@@ -777,7 +761,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Candidates and Criteria are optional. With no Criteria, the standard UOB rubric is used.</t>
+          <t>Criteria is optional. With no Criteria, the standard UOB rubric is used.</t>
         </is>
       </c>
     </row>
@@ -1561,101 +1545,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Candidate name *</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Role applied for</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Candidate One</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>c1@example.com</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>+6580000001</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>Analyst</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Candidate Two</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>c2@example.com</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>+6580000002</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Analyst</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
LAP rubric: 1-5 ratings with comments, Support for LAP, HR review redesign, stored PDF reports
- Setup Excel: Rubric sheet (Dimension, Descriptor, Score 1/3/5) and Event
  'Support question'; with no rubric the LAP rubric is used
- Judges rate each dimension 1-5 with a required comment and answer
  Support for LAP (Yes/No); submit is refused until all are filled in
- Review page: average out of 5, support counts, radar tinted rose/sand/sage,
  each dimension's scores and comments, HR decision and comments only
- PDF report made on the server when HR submits and stored with the
  decision; download per candidate or a day's reports as a zip
- Results and Excel show the average rating, support counts and raw
  ratings with comments
- Migration: rating scale, support question, min score, scorecard support,
  decision_reports

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qkgbu6zx8nSF6qinJQFGfA
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/event-setup-template.xlsx
+++ b/apps/web/public/templates/event-setup-template.xlsx
@@ -12,7 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day template" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Judges" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Availability" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rubric" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criteria" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -95,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -114,6 +115,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -211,6 +215,11 @@
         <t>Comma-separated. Each must already have a login (Users &amp; roles); they become admins of this event.</t>
       </text>
     </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Asked of every judge as Yes / No, e.g. Support for LAP. Leave blank for none.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -301,6 +310,41 @@
 </file>
 
 <file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Template</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>One row per dimension. Judges rate each 1 to 5 and must comment on each.</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>What the dimension is about. Shown to judges.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>What a 1 looks like. 2 sits between 1 and 3.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>What a 3 looks like. 4 sits between 3 and 5.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>What a 5 looks like.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>Template</author>
@@ -624,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -759,9 +803,33 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Criteria is optional. With no Criteria, the standard UOB rubric is used.</t>
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Rubric</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>The Rubric sheet holds the interview rubric: each dimension is rated 1 to 5 with a comment, and the candidate's score is the average rating out of 5. It comes filled in with the LAP rubric; edit it for another programme.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Support question on the Event sheet (e.g. Support for LAP) is asked of every judge as Yes / No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Criteria is an alternative points rubric (categories adding up to 100). Use either Rubric or Criteria, not both. With neither, the LAP rubric is used.</t>
         </is>
       </c>
     </row>
@@ -776,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -784,6 +852,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -812,6 +881,11 @@
           <t>Admin emails</t>
         </is>
       </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Support question</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -835,6 +909,11 @@
       <c r="E2" s="6" t="inlineStr">
         <is>
           <t>admin@example.com</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Support for LAP</t>
         </is>
       </c>
     </row>
@@ -1545,6 +1624,190 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Dimension *</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Descriptor</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Score: 1 (Low) *</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Score: 3 (Moderate) *</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Score: 5 (High) *</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Career Aspirations</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Clarity and ambition regarding future roles and career trajectory</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>No clear career goals; lacks interest in leadership or generalist roles.</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Expresses some interest in leadership but lacks clarity or commitment to generalist path.</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>Strong aspiration for senior leadership; clearly articulates interest in generalist roles and long-term growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Drive and Motivation</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Energy, initiative, and commitment to personal and organizational goals</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Passive attitude; limited examples of initiative or ownership.</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Shows moderate drive; some examples of taking initiative or leading efforts.</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Highly driven; consistently demonstrates ownership, resilience, and proactive leadership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Mobility &amp; Rotation Readiness</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Willingness and preparedness for new roles or rotations</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Unwilling to relocate or rotate; prefers stability.</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Open to some mobility; hesitant about full rotation model.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Fully open to geographic and functional rotations; embraces diverse experiences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Learning Agility &amp; Adaptability</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Ability to learn quickly and adapt to new situations</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Resistant to change; struggles with unfamiliar situations.</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>Some adaptability; has handled change with mixed success.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Highly agile; thrives in new environments and learns quickly from feedback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Enterprise Perspective</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Understanding and acting for the broader organization</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Narrow focus on own function; lacks cross-functional awareness.</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Some awareness of broader business; limited cross-functional experience.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Strong enterprise mindset; demonstrates strategic thinking and cross-functional collaboration.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Finer scores (e.g. 3.75) and per-dimension comment rules
- Setup Excel: Event 'Score step' (1, 0.5, 0.25 or 0.1; default 0.25) and
  Rubric 'Comment required' (Y/N per dimension; default Y)
- Judges tap a number; that button opens into a slider for the steps above
  it (3.00 to 3.75). Comments marked required or optional per dimension
- Scores stored as decimals; the server checks each score is on the step
- Migration: criterion_scores.score and scorecards.total_score to double
  precision, score_increment to DECIMAL(4,2); whole-number data converts as is

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qkgbu6zx8nSF6qinJQFGfA
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/event-setup-template.xlsx
+++ b/apps/web/public/templates/event-setup-template.xlsx
@@ -220,6 +220,11 @@
         <t>Asked of every judge as Yes / No, e.g. Support for LAP. Leave blank for none.</t>
       </text>
     </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>How finely judges can rate: 1 (whole numbers), 0.5, 0.25 (e.g. 3.75) or 0.1. Default 0.25.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -338,6 +343,11 @@
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>What a 5 looks like.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Y: judges must comment on this dimension. N: comment optional. Default Y.</t>
       </text>
     </comment>
   </commentList>
@@ -668,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -828,6 +838,20 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Score step on the Event sheet sets how finely judges can rate: 0.25 lets a judge give 3.75. Judges tap a number, then fine-tune it with the slider that appears in that button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Comment required on the Rubric sheet: Y makes the comment for that dimension mandatory, N makes it optional. Blank means Y.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Criteria is an alternative points rubric (categories adding up to 100). Use either Rubric or Criteria, not both. With neither, the LAP rubric is used.</t>
         </is>
@@ -844,7 +868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -853,6 +877,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -886,6 +911,11 @@
           <t>Support question</t>
         </is>
       </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Score step</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -915,6 +945,9 @@
         <is>
           <t>Support for LAP</t>
         </is>
+      </c>
+      <c r="G2" s="6" t="n">
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>
@@ -1624,7 +1657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1632,6 +1665,7 @@
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1660,6 +1694,11 @@
           <t>Score: 5 (High) *</t>
         </is>
       </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Comment required</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -1687,6 +1726,11 @@
           <t>Strong aspiration for senior leadership; clearly articulates interest in generalist roles and long-term growth.</t>
         </is>
       </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1714,6 +1758,11 @@
           <t>Highly driven; consistently demonstrates ownership, resilience, and proactive leadership.</t>
         </is>
       </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -1741,6 +1790,11 @@
           <t>Fully open to geographic and functional rotations; embraces diverse experiences.</t>
         </is>
       </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1768,6 +1822,11 @@
           <t>Highly agile; thrives in new environments and learns quickly from feedback.</t>
         </is>
       </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1795,8 +1854,18 @@
           <t>Strong enterprise mindset; demonstrates strategic thinking and cross-functional collaboration.</t>
         </is>
       </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>

<commit_message>
Score step set per dimension on the Rubric sheet
Moves 'Score step' from the Event sheet to the Rubric sheet, next to
'Comment required', so each dimension's scoring rules sit together.
Blank means 0.25. Judges never choose the step.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qkgbu6zx8nSF6qinJQFGfA
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/event-setup-template.xlsx
+++ b/apps/web/public/templates/event-setup-template.xlsx
@@ -220,11 +220,6 @@
         <t>Asked of every judge as Yes / No, e.g. Support for LAP. Leave blank for none.</t>
       </text>
     </comment>
-    <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>How finely judges can rate: 1 (whole numbers), 0.5, 0.25 (e.g. 3.75) or 0.1. Default 0.25.</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -348,6 +343,11 @@
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Y: judges must comment on this dimension. N: comment optional. Default Y.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>How finely judges can rate this dimension: 1 (whole numbers), 0.5, 0.25 (e.g. 3.75) or 0.1. Default 0.25.</t>
       </text>
     </comment>
   </commentList>
@@ -678,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -839,19 +839,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Score step on the Event sheet sets how finely judges can rate: 0.25 lets a judge give 3.75. Judges tap a number, then fine-tune it with the slider that appears in that button.</t>
+          <t>Each Rubric row also sets that dimension's scoring rules. Comment required: Y makes the comment mandatory, N optional (blank = Y). Score step: how finely judges can rate, 1, 0.5, 0.25 or 0.1 (blank = 0.25); with 0.25 a judge can give 3.75.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Comment required on the Rubric sheet: Y makes the comment for that dimension mandatory, N makes it optional. Blank means Y.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Criteria is an alternative points rubric (categories adding up to 100). Use either Rubric or Criteria, not both. With neither, the LAP rubric is used.</t>
         </is>
@@ -868,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -877,7 +870,6 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -911,11 +903,6 @@
           <t>Support question</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Score step</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -945,9 +932,6 @@
         <is>
           <t>Support for LAP</t>
         </is>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>0.25</v>
       </c>
     </row>
   </sheetData>
@@ -1657,7 +1641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1666,6 +1650,7 @@
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1699,6 +1684,11 @@
           <t>Comment required</t>
         </is>
       </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>Score step</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -1731,6 +1721,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G2" s="8" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -1763,6 +1756,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G3" s="8" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -1795,6 +1791,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G4" s="8" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1827,6 +1826,9 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G5" s="8" t="n">
+        <v>0.25</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1859,11 +1861,17 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G6" s="8" t="n">
+        <v>0.25</v>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1,0.5,0.25,0.1"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>